<commit_message>
Switch model to LAC countries and add DSPTRN dispatch technology
- Replace South Asian country set (BGD/BTN/IND/NPL/LKA/MDV) with 19 Latin American countries
- Add DSPTRN dispatch technology and enable_dsptrn flag for 4-tier ELC routing (ELC00/01/02/03)
- Add force_empty_max_capacity_investment_pwr config flag
- Consolidate set DataFrames (STORAGE, TECHNOLOGY, FUEL) during region merging
- Update template_generation to support multi-entry list format with centerpoints
- Regenerate all A1 outputs and A2 otoole params for new country configuration
</commit_message>
<xml_diff>
--- a/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_Demand_COMPLETED.xlsx
+++ b/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_Demand_COMPLETED.xlsx
@@ -166,118 +166,118 @@
     <t>Demand</t>
   </si>
   <si>
-    <t>ELCARGXX02</t>
+    <t>ELCARGXX03</t>
   </si>
   <si>
-    <t>ELCBOLXX02</t>
+    <t>ELCBOLXX03</t>
   </si>
   <si>
-    <t>ELCBRAXX02</t>
+    <t>ELCBRAXX03</t>
   </si>
   <si>
-    <t>ELCBRBXX02</t>
+    <t>ELCBRBXX03</t>
   </si>
   <si>
-    <t>ELCCHLXX02</t>
+    <t>ELCCHLXX03</t>
   </si>
   <si>
-    <t>ELCCOLXX02</t>
+    <t>ELCCOLXX03</t>
   </si>
   <si>
-    <t>ELCCRIXX02</t>
+    <t>ELCCRIXX03</t>
   </si>
   <si>
-    <t>ELCDOMXX02</t>
+    <t>ELCDOMXX03</t>
   </si>
   <si>
-    <t>ELCECUXX02</t>
+    <t>ELCECUXX03</t>
   </si>
   <si>
-    <t>ELCGTMXX02</t>
+    <t>ELCGTMXX03</t>
   </si>
   <si>
-    <t>ELCHNDXX02</t>
+    <t>ELCHNDXX03</t>
   </si>
   <si>
-    <t>ELCHTIXX02</t>
+    <t>ELCHTIXX03</t>
   </si>
   <si>
-    <t>ELCMEXXX02</t>
+    <t>ELCMEXXX03</t>
   </si>
   <si>
-    <t>ELCNICXX02</t>
+    <t>ELCNICXX03</t>
   </si>
   <si>
-    <t>ELCPANXX02</t>
+    <t>ELCPANXX03</t>
   </si>
   <si>
-    <t>ELCPERXX02</t>
+    <t>ELCPERXX03</t>
   </si>
   <si>
-    <t>ELCPRYXX02</t>
+    <t>ELCPRYXX03</t>
   </si>
   <si>
-    <t>ELCSLVXX02</t>
+    <t>ELCSLVXX03</t>
   </si>
   <si>
-    <t>ELCURYXX02</t>
+    <t>ELCURYXX03</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Argentina</t>
+    <t>Output demand of dispatch-readys in Argentina</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Bolivia</t>
+    <t>Output demand of dispatch-readys in Bolivia</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Brazil</t>
+    <t>Output demand of dispatch-readys in Brazil</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Barbados</t>
+    <t>Output demand of dispatch-readys in Barbados</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Chile</t>
+    <t>Output demand of dispatch-readys in Chile</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Colombia</t>
+    <t>Output demand of dispatch-readys in Colombia</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Costa Rica</t>
+    <t>Output demand of dispatch-readys in Costa Rica</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Dominican Republic</t>
+    <t>Output demand of dispatch-readys in Dominican Republic</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Ecuador</t>
+    <t>Output demand of dispatch-readys in Ecuador</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Guatemala</t>
+    <t>Output demand of dispatch-readys in Guatemala</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Honduras</t>
+    <t>Output demand of dispatch-readys in Honduras</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Haiti</t>
+    <t>Output demand of dispatch-readys in Haiti</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Mexico</t>
+    <t>Output demand of dispatch-readys in Mexico</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Nicaragua</t>
+    <t>Output demand of dispatch-readys in Nicaragua</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Panama</t>
+    <t>Output demand of dispatch-readys in Panama</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Peru</t>
+    <t>Output demand of dispatch-readys in Peru</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Paraguay</t>
+    <t>Output demand of dispatch-readys in Paraguay</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in El Salvador</t>
+    <t>Output demand of dispatch-readys in El Salvador</t>
   </si>
   <si>
-    <t>Output demand of transmission lines in Uruguay</t>
+    <t>Output demand of dispatch-readys in Uruguay</t>
   </si>
   <si>
     <t>not needed</t>

</xml_diff>

<commit_message>
Update A1/A2 outputs, OG inputs, and config files
</commit_message>
<xml_diff>
--- a/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_Demand_COMPLETED.xlsx
+++ b/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_Demand_COMPLETED.xlsx
@@ -166,118 +166,118 @@
     <t>Demand</t>
   </si>
   <si>
-    <t>ELCARGXX03</t>
+    <t>ELCARGXX02</t>
   </si>
   <si>
-    <t>ELCBOLXX03</t>
+    <t>ELCBOLXX02</t>
   </si>
   <si>
-    <t>ELCBRAXX03</t>
+    <t>ELCBRAXX02</t>
   </si>
   <si>
-    <t>ELCBRBXX03</t>
+    <t>ELCBRBXX02</t>
   </si>
   <si>
-    <t>ELCCHLXX03</t>
+    <t>ELCCHLXX02</t>
   </si>
   <si>
-    <t>ELCCOLXX03</t>
+    <t>ELCCOLXX02</t>
   </si>
   <si>
-    <t>ELCCRIXX03</t>
+    <t>ELCCRIXX02</t>
   </si>
   <si>
-    <t>ELCDOMXX03</t>
+    <t>ELCDOMXX02</t>
   </si>
   <si>
-    <t>ELCECUXX03</t>
+    <t>ELCECUXX02</t>
   </si>
   <si>
-    <t>ELCGTMXX03</t>
+    <t>ELCGTMXX02</t>
   </si>
   <si>
-    <t>ELCHNDXX03</t>
+    <t>ELCHNDXX02</t>
   </si>
   <si>
-    <t>ELCHTIXX03</t>
+    <t>ELCHTIXX02</t>
   </si>
   <si>
-    <t>ELCMEXXX03</t>
+    <t>ELCMEXXX02</t>
   </si>
   <si>
-    <t>ELCNICXX03</t>
+    <t>ELCNICXX02</t>
   </si>
   <si>
-    <t>ELCPANXX03</t>
+    <t>ELCPANXX02</t>
   </si>
   <si>
-    <t>ELCPERXX03</t>
+    <t>ELCPERXX02</t>
   </si>
   <si>
-    <t>ELCPRYXX03</t>
+    <t>ELCPRYXX02</t>
   </si>
   <si>
-    <t>ELCSLVXX03</t>
+    <t>ELCSLVXX02</t>
   </si>
   <si>
-    <t>ELCURYXX03</t>
+    <t>ELCURYXX02</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Argentina</t>
+    <t>Output demand of transmission lines in Argentina</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Bolivia</t>
+    <t>Output demand of transmission lines in Bolivia</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Brazil</t>
+    <t>Output demand of transmission lines in Brazil</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Barbados</t>
+    <t>Output demand of transmission lines in Barbados</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Chile</t>
+    <t>Output demand of transmission lines in Chile</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Colombia</t>
+    <t>Output demand of transmission lines in Colombia</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Costa Rica</t>
+    <t>Output demand of transmission lines in Costa Rica</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Dominican Republic</t>
+    <t>Output demand of transmission lines in Dominican Republic</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Ecuador</t>
+    <t>Output demand of transmission lines in Ecuador</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Guatemala</t>
+    <t>Output demand of transmission lines in Guatemala</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Honduras</t>
+    <t>Output demand of transmission lines in Honduras</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Haiti</t>
+    <t>Output demand of transmission lines in Haiti</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Mexico</t>
+    <t>Output demand of transmission lines in Mexico</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Nicaragua</t>
+    <t>Output demand of transmission lines in Nicaragua</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Panama</t>
+    <t>Output demand of transmission lines in Panama</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Peru</t>
+    <t>Output demand of transmission lines in Peru</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Paraguay</t>
+    <t>Output demand of transmission lines in Paraguay</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in El Salvador</t>
+    <t>Output demand of transmission lines in El Salvador</t>
   </si>
   <si>
-    <t>Output demand of dispatch-readys in Uruguay</t>
+    <t>Output demand of transmission lines in Uruguay</t>
   </si>
   <si>
     <t>not needed</t>

</xml_diff>